<commit_message>
docs(registros): alinha equipe (GP Abraão, Cézar TL/DevOps/Arq, devs Raony/Mateus/Lucas, QA Caroline, GQA Jonathan)
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mps-nivel-c/oficial/04_registros/AASP_Andamento-Processuais/GEST-AASPAP01_Planilha-de-Gestao-do-Projeto.xlsx
+++ b/mps-nivel-c/oficial/04_registros/AASP_Andamento-Processuais/GEST-AASPAP01_Planilha-de-Gestao-do-Projeto.xlsx
@@ -866,7 +866,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -906,7 +905,7 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Cezar Hiraki Velazquez</t>
+          <t>Abraão Oliveira</t>
         </is>
       </c>
     </row>
@@ -982,7 +981,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="47" t="inlineStr">
         <is>
@@ -1056,7 +1054,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="47" t="inlineStr">
         <is>
@@ -1350,7 +1347,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
@@ -1399,8 +1395,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="47" t="inlineStr">
         <is>
@@ -1705,7 +1699,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="47" t="inlineStr">
         <is>
@@ -2037,7 +2030,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
     <row r="37">
       <c r="A37" s="47" t="inlineStr">
         <is>
@@ -2925,8 +2917,6 @@
       <c r="I18" s="6" t="n"/>
       <c r="J18" s="7" t="n"/>
     </row>
-    <row r="19"/>
-    <row r="20"/>
     <row r="21" ht="19.95" customHeight="1" s="38">
       <c r="A21" s="50" t="inlineStr">
         <is>
@@ -3122,7 +3112,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -3426,7 +3415,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="47" t="inlineStr">
         <is>
@@ -5458,7 +5446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="28" customWidth="1" style="38" min="1" max="1"/>
@@ -5483,7 +5471,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -5526,12 +5513,12 @@
     <row r="6" ht="26.4" customHeight="1" s="38">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t>Cezar Hiraki · Tech Lead / Arquiteto de Software</t>
+          <t>Abraão Oliveira · Gerente de Projeto</t>
         </is>
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Planejamento técnico, arquitetura da solução e decisões de design</t>
+          <t>Gestão das entregas, planejamento e aceite</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
@@ -5551,19 +5538,19 @@
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
-          <t>Ponto focal técnico Timeware — todas as fases</t>
+          <t>Ponto focal de gestão — todas as fases</t>
         </is>
       </c>
     </row>
     <row r="7" ht="39.6" customHeight="1" s="38">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>Raony Chagas · Desenvolvedor Sênior (Principal)</t>
+          <t>Cézar Hiraki Velázquez · Tech Lead / DevOps / Arquiteto</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>Implementação das refatorações: webhook, CapturaServer, lógica de movimentações</t>
+          <t>Planejamento técnico, arquitetura, CI/CD e GMUD</t>
         </is>
       </c>
       <c r="C7" s="15" t="inlineStr">
@@ -5583,24 +5570,24 @@
       </c>
       <c r="F7" s="16" t="inlineStr">
         <is>
-          <t>Responsável técnico principal em todas as fases</t>
+          <t>Ponto focal técnico Timeware</t>
         </is>
       </c>
     </row>
     <row r="8" ht="39.6" customHeight="1" s="38">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>Mateus Veloso · Desenvolvedor (Suporte)</t>
+          <t>Raony Chagas · Desenvolvedor Sênior (Principal)</t>
         </is>
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>Suporte ao desenvolvimento de endpoints, fluxo de parceiras e correções</t>
+          <t>Refatorações: webhook, CapturaServer, movimentações</t>
         </is>
       </c>
       <c r="C8" s="24" t="inlineStr">
         <is>
-          <t>❌ Não</t>
+          <t>✅ Sim</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
@@ -5610,24 +5597,24 @@
       </c>
       <c r="E8" s="13" t="inlineStr">
         <is>
-          <t>100% (Fases 3–4)</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="F8" s="13" t="inlineStr">
         <is>
-          <t>Incorporado a partir de Abr/2026</t>
+          <t>Responsável técnico principal</t>
         </is>
       </c>
     </row>
     <row r="9" ht="26.4" customHeight="1" s="38">
       <c r="A9" s="16" t="inlineStr">
         <is>
-          <t>Caroline Sousa · Analista de QA</t>
+          <t>Mateus Veloso · Desenvolvedor (Suporte)</t>
         </is>
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>Execução de testes de fluxo e validação dos critérios de aceite</t>
+          <t>Suporte ao desenvolvimento, fluxo de parceiras e correções</t>
         </is>
       </c>
       <c r="C9" s="24" t="inlineStr">
@@ -5637,17 +5624,17 @@
       </c>
       <c r="D9" s="15" t="inlineStr">
         <is>
-          <t>✅ Sim (Fase 4)</t>
+          <t>✅ Sim</t>
         </is>
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
-          <t>Parcial (Fase 4)</t>
+          <t>100% (Fases 3–4)</t>
         </is>
       </c>
       <c r="F9" s="16" t="inlineStr">
         <is>
-          <t>Mai/2026 – Jun/2026</t>
+          <t>Incorporado a partir de Abr/2026</t>
         </is>
       </c>
     </row>
@@ -5659,7 +5646,7 @@
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>Provisionamento de ambientes, GMUD e deploy em produção</t>
+          <t>Provisionamento de ambientes, GMUD e deploy</t>
         </is>
       </c>
       <c r="C10" s="15" t="inlineStr">
@@ -5683,95 +5670,143 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Caroline Sousa · Analista de QA</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Execução de testes de fluxo e validação dos critérios de aceite</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>❌ Não</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>✅ Sim (Fase 4)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Parcial (Fase 4)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Mai/2026 – Jun/2026</t>
+        </is>
+      </c>
+    </row>
     <row r="12">
-      <c r="A12" s="47" t="inlineStr">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Jonathan Barbosa · Auditor GQA (independente)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Verificação de aderência ao processo MPS-SW</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>✅ Sim</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Não participa da execução</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14" ht="39.6" customHeight="1" s="38">
+      <c r="A14" s="47" t="inlineStr">
         <is>
           <t>PARTES INTERESSADAS — CLIENTE (AASP — Associação dos Advogados de São Paulo)</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="14" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>Nome</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>Papel / Função</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
+      <c r="C15" s="14" t="inlineStr">
         <is>
           <t>Envolvimento</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
+      <c r="D15" s="14" t="inlineStr">
         <is>
           <t>Fases 1–2</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
+      <c r="E15" s="14" t="inlineStr">
         <is>
           <t>Fases 3–4</t>
         </is>
       </c>
-      <c r="F13" s="14" t="inlineStr">
+      <c r="F15" s="14" t="inlineStr">
         <is>
           <t>Ponto de contato principal</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="39.6" customHeight="1" s="38">
-      <c r="A14" s="13" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
         <is>
           <t>Marcos Correa Fernandez Turnes · Representante do Cliente (AASP)</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>Product Owner / Decisor</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="C16" s="13" t="inlineStr">
         <is>
           <t>Validação dos requisitos, homologação e aceite das entregas</t>
         </is>
       </c>
-      <c r="D14" s="15" t="inlineStr">
+      <c r="D16" s="15" t="inlineStr">
         <is>
           <t>✅ Sim</t>
         </is>
       </c>
-      <c r="E14" s="15" t="inlineStr">
+      <c r="E16" s="15" t="inlineStr">
         <is>
           <t>✅ Sim</t>
         </is>
       </c>
-      <c r="F14" s="13" t="inlineStr">
+      <c r="F16" s="13" t="inlineStr">
         <is>
           <t>Aceite formal das fases</t>
         </is>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16">
-      <c r="A16" s="1" t="n"/>
-      <c r="B16" s="1" t="n"/>
-      <c r="C16" s="1" t="n"/>
-      <c r="D16" s="1" t="n"/>
-      <c r="E16" s="1" t="n"/>
-      <c r="F16" s="1" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="n"/>
-      <c r="B17" s="1" t="n"/>
-      <c r="C17" s="1" t="n"/>
-      <c r="D17" s="1" t="n"/>
-      <c r="E17" s="1" t="n"/>
-      <c r="F17" s="1" t="n"/>
-    </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="1" t="n"/>
       <c r="B18" s="1" t="n"/>
@@ -5779,6 +5814,22 @@
       <c r="D18" s="1" t="n"/>
       <c r="E18" s="1" t="n"/>
       <c r="F18" s="1" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n"/>
+      <c r="B19" s="1" t="n"/>
+      <c r="C19" s="1" t="n"/>
+      <c r="D19" s="1" t="n"/>
+      <c r="E19" s="1" t="n"/>
+      <c r="F19" s="1" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n"/>
+      <c r="B20" s="1" t="n"/>
+      <c r="C20" s="1" t="n"/>
+      <c r="D20" s="1" t="n"/>
+      <c r="E20" s="1" t="n"/>
+      <c r="F20" s="1" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -5822,7 +5873,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -6142,7 +6192,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="47" t="inlineStr">
         <is>
@@ -6358,7 +6407,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="47" t="inlineStr">
         <is>
@@ -6544,7 +6592,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -7100,7 +7147,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="57" t="inlineStr">
         <is>
@@ -7186,7 +7232,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(registros): tabelas de equipe idênticas (roster canônico) em TAP/INTAKE; Lucas como Desenvolvedor
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mps-nivel-c/oficial/04_registros/AASP_Andamento-Processuais/GEST-AASPAP01_Planilha-de-Gestao-do-Projeto.xlsx
+++ b/mps-nivel-c/oficial/04_registros/AASP_Andamento-Processuais/GEST-AASPAP01_Planilha-de-Gestao-do-Projeto.xlsx
@@ -5471,6 +5471,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -5641,7 +5642,7 @@
     <row r="10" ht="26.4" customHeight="1" s="38">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>Lucas Batista · DevOps / Infraestrutura</t>
+          <t>Lucas Batista · Desenvolvedor</t>
         </is>
       </c>
       <c r="B10" s="13" t="inlineStr">
@@ -5703,34 +5704,9 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>Jonathan Barbosa · Auditor GQA (independente)</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Verificação de aderência ao processo MPS-SW</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>✅ Sim</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Auditoria</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Não participa da execução</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(registros): corrige achados de auditoria (N1 papel GP, N2/M1 citações INTAKE, M2 CR consolidado, M4 banner)
- N1: 'Tech Lead acumula DevOps e Arquiteto' (Abraão é o GP)
- N2/M1: remove citações ao INTAKE (removido do repo) e a data 14/06; troca fonte p/ GEST/registros
- M2: referências a CR-*-002 apontam para o CR consolidado (-001)
- M4: banner com código correto e Versão 1.0

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mps-nivel-c/oficial/04_registros/AASP_Andamento-Processuais/GEST-AASPAP01_Planilha-de-Gestao-do-Projeto.xlsx
+++ b/mps-nivel-c/oficial/04_registros/AASP_Andamento-Processuais/GEST-AASPAP01_Planilha-de-Gestao-do-Projeto.xlsx
@@ -866,6 +866,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -981,6 +982,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="47" t="inlineStr">
         <is>
@@ -1054,6 +1056,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="47" t="inlineStr">
         <is>
@@ -1347,6 +1350,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
@@ -1395,6 +1399,8 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="47" t="inlineStr">
         <is>
@@ -1699,6 +1705,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="47" t="inlineStr">
         <is>
@@ -2030,6 +2037,7 @@
         </is>
       </c>
     </row>
+    <row r="36"/>
     <row r="37">
       <c r="A37" s="47" t="inlineStr">
         <is>
@@ -2917,6 +2925,8 @@
       <c r="I18" s="6" t="n"/>
       <c r="J18" s="7" t="n"/>
     </row>
+    <row r="19"/>
+    <row r="20"/>
     <row r="21" ht="19.95" customHeight="1" s="38">
       <c r="A21" s="50" t="inlineStr">
         <is>
@@ -3112,6 +3122,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -3415,6 +3426,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="47" t="inlineStr">
         <is>
@@ -5849,6 +5861,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -6168,6 +6181,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="47" t="inlineStr">
         <is>
@@ -6383,6 +6397,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="47" t="inlineStr">
         <is>
@@ -6481,7 +6496,7 @@
     <row r="21" ht="118.8" customHeight="1" s="38">
       <c r="A21" s="16" t="inlineStr">
         <is>
-          <t>CR-AASPAP01-002</t>
+          <t>CR-AASPAP01-001</t>
         </is>
       </c>
       <c r="B21" s="16" t="inlineStr">
@@ -6568,6 +6583,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -6993,7 +7009,7 @@
     <row r="2">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Referência: CR-AASPAP01-001 · CR-AASPAP01-002 · REG-AASPAP01-001 §3.5</t>
+          <t>Referência: CR-AASPAP01-001 · CR-AASPAP01-001 · REG-AASPAP01-001 §3.5</t>
         </is>
       </c>
     </row>
@@ -7084,7 +7100,7 @@
     <row r="5">
       <c r="A5" s="55" t="inlineStr">
         <is>
-          <t>CR-AASPAP01-002</t>
+          <t>CR-AASPAP01-001</t>
         </is>
       </c>
       <c r="B5" s="55" t="inlineStr">
@@ -7123,6 +7139,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="57" t="inlineStr">
         <is>
@@ -7208,6 +7225,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: corrige contradições da auditoria (status em execução, v241 contenção pré-go-live, GP no PLA, horas 586/~624, T-39/T-19, CR AP separado 001+002, BL-HOTFIX, RF09->T-19)
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mps-nivel-c/oficial/04_registros/AASP_Andamento-Processuais/GEST-AASPAP01_Planilha-de-Gestao-do-Projeto.xlsx
+++ b/mps-nivel-c/oficial/04_registros/AASP_Andamento-Processuais/GEST-AASPAP01_Planilha-de-Gestao-do-Projeto.xlsx
@@ -866,7 +866,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -982,7 +981,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="47" t="inlineStr">
         <is>
@@ -1056,7 +1054,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="47" t="inlineStr">
         <is>
@@ -1350,7 +1347,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
@@ -1399,8 +1395,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="47" t="inlineStr">
         <is>
@@ -1705,7 +1699,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="47" t="inlineStr">
         <is>
@@ -2037,7 +2030,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
     <row r="37">
       <c r="A37" s="47" t="inlineStr">
         <is>
@@ -2925,8 +2917,6 @@
       <c r="I18" s="6" t="n"/>
       <c r="J18" s="7" t="n"/>
     </row>
-    <row r="19"/>
-    <row r="20"/>
     <row r="21" ht="19.95" customHeight="1" s="38">
       <c r="A21" s="50" t="inlineStr">
         <is>
@@ -3122,7 +3112,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -3426,7 +3415,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="47" t="inlineStr">
         <is>
@@ -4707,7 +4695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" style="38" min="1" max="1"/>
@@ -5437,9 +5425,46 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="56" t="inlineStr">
-        <is>
-          <t>18 tarefas — 18 concluídas</t>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>T-19</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Tratamento de NUP inválido (status 8 / resposta 10) por instância</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Mai/2026</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Jun/2026</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>RF09</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Concluída</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="56" t="inlineStr">
+        <is>
+          <t>19 tarefas — 19 concluídas</t>
         </is>
       </c>
     </row>
@@ -5483,7 +5508,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -5722,7 +5746,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="39.6" customHeight="1" s="38">
       <c r="A14" s="47" t="inlineStr">
         <is>
@@ -5794,7 +5817,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="1" t="n"/>
       <c r="B18" s="1" t="n"/>
@@ -5861,7 +5883,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -6181,7 +6202,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="47" t="inlineStr">
         <is>
@@ -6397,7 +6417,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="47" t="inlineStr">
         <is>
@@ -6583,7 +6602,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -7139,7 +7157,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="57" t="inlineStr">
         <is>
@@ -7225,7 +7242,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: 2ª rodada de correções de auditoria (601->586/+~6%, CR AP 001+002 na aba, CR-CNJ-002, RF12 fase F2, RF09 cross-repo, BL-EPROC v230, GCO 4 tags, inversões de data)
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mps-nivel-c/oficial/04_registros/AASP_Andamento-Processuais/GEST-AASPAP01_Planilha-de-Gestao-do-Projeto.xlsx
+++ b/mps-nivel-c/oficial/04_registros/AASP_Andamento-Processuais/GEST-AASPAP01_Planilha-de-Gestao-do-Projeto.xlsx
@@ -866,6 +866,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -981,6 +982,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="47" t="inlineStr">
         <is>
@@ -1054,6 +1056,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="47" t="inlineStr">
         <is>
@@ -1347,6 +1350,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
@@ -1395,6 +1399,8 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="47" t="inlineStr">
         <is>
@@ -1699,6 +1705,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="47" t="inlineStr">
         <is>
@@ -2030,6 +2037,7 @@
         </is>
       </c>
     </row>
+    <row r="36"/>
     <row r="37">
       <c r="A37" s="47" t="inlineStr">
         <is>
@@ -2917,6 +2925,8 @@
       <c r="I18" s="6" t="n"/>
       <c r="J18" s="7" t="n"/>
     </row>
+    <row r="19"/>
+    <row r="20"/>
     <row r="21" ht="19.95" customHeight="1" s="38">
       <c r="A21" s="50" t="inlineStr">
         <is>
@@ -3112,6 +3122,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -3415,6 +3426,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="47" t="inlineStr">
         <is>
@@ -5508,6 +5520,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -5746,6 +5759,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="39.6" customHeight="1" s="38">
       <c r="A14" s="47" t="inlineStr">
         <is>
@@ -5817,6 +5831,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="1" t="n"/>
       <c r="B18" s="1" t="n"/>
@@ -5883,6 +5898,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -6202,6 +6218,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="47" t="inlineStr">
         <is>
@@ -6417,6 +6434,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="47" t="inlineStr">
         <is>
@@ -6602,6 +6620,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -7027,7 +7046,7 @@
     <row r="2">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Referência: CR-AASPAP01-001 · CR-AASPAP01-001 · REG-AASPAP01-001 §3.5</t>
+          <t>Referência: CR-AASPAP01-001 · CR-AASPAP01-002 · REG-AASPAP01-001 §3.5</t>
         </is>
       </c>
     </row>
@@ -7118,7 +7137,7 @@
     <row r="5">
       <c r="A5" s="55" t="inlineStr">
         <is>
-          <t>CR-AASPAP01-001</t>
+          <t>CR-AASPAP01-002</t>
         </is>
       </c>
       <c r="B5" s="55" t="inlineStr">
@@ -7157,6 +7176,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="57" t="inlineStr">
         <is>
@@ -7242,6 +7262,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: saneamento de auditoria (Fase 6 em andamento, RNF06 projetado, captcha->RNF01, T-14+RF08, T-19 fim, nota dev x merge, revisão por pares)
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mps-nivel-c/oficial/04_registros/AASP_Andamento-Processuais/GEST-AASPAP01_Planilha-de-Gestao-do-Projeto.xlsx
+++ b/mps-nivel-c/oficial/04_registros/AASP_Andamento-Processuais/GEST-AASPAP01_Planilha-de-Gestao-do-Projeto.xlsx
@@ -866,7 +866,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -982,7 +981,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="47" t="inlineStr">
         <is>
@@ -1056,7 +1054,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="47" t="inlineStr">
         <is>
@@ -1350,7 +1347,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
@@ -1399,8 +1395,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="47" t="inlineStr">
         <is>
@@ -1705,7 +1699,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="47" t="inlineStr">
         <is>
@@ -2037,7 +2030,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
     <row r="37">
       <c r="A37" s="47" t="inlineStr">
         <is>
@@ -2925,8 +2917,6 @@
       <c r="I18" s="6" t="n"/>
       <c r="J18" s="7" t="n"/>
     </row>
-    <row r="19"/>
-    <row r="20"/>
     <row r="21" ht="19.95" customHeight="1" s="38">
       <c r="A21" s="50" t="inlineStr">
         <is>
@@ -3122,7 +3112,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -3426,7 +3415,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="47" t="inlineStr">
         <is>
@@ -5279,7 +5267,7 @@
       </c>
       <c r="F17" s="55" t="inlineStr">
         <is>
-          <t>RF07, RF11</t>
+          <t>RF07, RF08, RF11</t>
         </is>
       </c>
       <c r="G17" s="55" t="inlineStr">
@@ -5454,7 +5442,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Jun/2026</t>
+          <t>Mai/2026</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -5520,7 +5508,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -5759,7 +5746,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="39.6" customHeight="1" s="38">
       <c r="A14" s="47" t="inlineStr">
         <is>
@@ -5831,7 +5817,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="1" t="n"/>
       <c r="B18" s="1" t="n"/>
@@ -5898,7 +5883,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -6218,7 +6202,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="47" t="inlineStr">
         <is>
@@ -6434,7 +6417,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="47" t="inlineStr">
         <is>
@@ -6620,7 +6602,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -7176,7 +7157,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="57" t="inlineStr">
         <is>
@@ -7262,7 +7242,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: 3ª rodada — fecha ALTA (RF07/RF08 cross-repo, encerramento 30/06, aderência ~88%, defeitos 10) + médias (T-20 AP, desvio +38h, v240 rótulo, GCO hotfix, resp F5)
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mps-nivel-c/oficial/04_registros/AASP_Andamento-Processuais/GEST-AASPAP01_Planilha-de-Gestao-do-Projeto.xlsx
+++ b/mps-nivel-c/oficial/04_registros/AASP_Andamento-Processuais/GEST-AASPAP01_Planilha-de-Gestao-do-Projeto.xlsx
@@ -4695,7 +4695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" style="38" min="1" max="1"/>
@@ -5462,9 +5462,46 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="56" t="inlineStr">
-        <is>
-          <t>19 tarefas — 19 concluídas</t>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>T-20</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Hotfix de contenção (homologação): nullabilidade em CapturaLogin sob carga — v241</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Jun/2026</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Jun/2026</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>RNF04</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Concluída</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="56" t="inlineStr">
+        <is>
+          <t>20 tarefas — 20 concluídas</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: resíduo de auditoria (BAIXA) — coerência de fases/CRs/tags
- AP GEST: linha Fase 5 (Implantação 🟡 Em andamento) no RESUMO POR PACOTE
- CNJ GEST: T-12 alinhada a RF02/US-03 (1ª instância EPROC + incidentes ESAJ)
- AP CR-002: escopo RF07-RF12 -> RF07-RF09, RF11, RF12 (RF10/CodigoFonteAPI e Fase 3)
- AP RAC: CR de Fase 4 -> CR-AASPAP01-002 (remove CodigoFonteAPI/Fase 3)
- CNJ GCO: evidencia de auditoria lista v230, v240 e v241

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mps-nivel-c/oficial/04_registros/AASP_Andamento-Processuais/GEST-AASPAP01_Planilha-de-Gestao-do-Projeto.xlsx
+++ b/mps-nivel-c/oficial/04_registros/AASP_Andamento-Processuais/GEST-AASPAP01_Planilha-de-Gestao-do-Projeto.xlsx
@@ -1054,6 +1054,28 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>Fase 5 — Implantação / Go-live</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Implantação em produção, homologação pré-go-live e estabilização</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Jun/2026</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>🟡 Em andamento</t>
+        </is>
+      </c>
+    </row>
     <row r="20">
       <c r="A20" s="47" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(registros): espelha AASP_CNJ e AASP_AndamentosProcessuais da cnj_andamentos (fonte de verdade)
Sobrepõe as duas pastas de oficial/04_registros com o conteúdo atual da branch
cnj_andamentos, tratada como ponto de verdade:
- AASP_CNJ: adiciona CR-AASPCNJ01-002 e evidências (swagger/postman/devops/schemas),
  atualiza os 18 docx + GEST; remove os .md-fonte, o 00_INDICE e o CAP
  (Registro de Capacitação) por não existirem na fonte de verdade.
- AASP_AndamentosProcessuais: adiciona CR-AASPAP01-002 e atualiza 13 docx/planilha.

https://claude.ai/code/session_01D9YHKrGanfZsACSZKYQDTp
</commit_message>
<xml_diff>
--- a/mps-nivel-c/oficial/04_registros/AASP_Andamento-Processuais/GEST-AASPAP01_Planilha-de-Gestao-do-Projeto.xlsx
+++ b/mps-nivel-c/oficial/04_registros/AASP_Andamento-Processuais/GEST-AASPAP01_Planilha-de-Gestao-do-Projeto.xlsx
@@ -866,7 +866,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -982,7 +981,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="47" t="inlineStr">
         <is>
@@ -1056,7 +1054,28 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>Fase 5 — Implantação / Go-live</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Implantação em produção, homologação pré-go-live e estabilização</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Jun/2026</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>🟡 Em andamento</t>
+        </is>
+      </c>
+    </row>
     <row r="20">
       <c r="A20" s="47" t="inlineStr">
         <is>
@@ -1350,7 +1369,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
@@ -1399,8 +1417,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="47" t="inlineStr">
         <is>
@@ -1705,7 +1721,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="47" t="inlineStr">
         <is>
@@ -2037,7 +2052,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
     <row r="37">
       <c r="A37" s="47" t="inlineStr">
         <is>
@@ -2925,8 +2939,6 @@
       <c r="I18" s="6" t="n"/>
       <c r="J18" s="7" t="n"/>
     </row>
-    <row r="19"/>
-    <row r="20"/>
     <row r="21" ht="19.95" customHeight="1" s="38">
       <c r="A21" s="50" t="inlineStr">
         <is>
@@ -3122,7 +3134,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -3426,7 +3437,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="47" t="inlineStr">
         <is>
@@ -4707,7 +4717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" style="38" min="1" max="1"/>
@@ -5279,7 +5289,7 @@
       </c>
       <c r="F17" s="55" t="inlineStr">
         <is>
-          <t>RF07, RF11</t>
+          <t>RF07, RF08, RF11</t>
         </is>
       </c>
       <c r="G17" s="55" t="inlineStr">
@@ -5437,9 +5447,83 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="56" t="inlineStr">
-        <is>
-          <t>18 tarefas — 18 concluídas</t>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>T-19</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Tratamento de NUP inválido (status 8 / resposta 10) por instância</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Mai/2026</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Mai/2026</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>RF09</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Concluída</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>T-20</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Hotfix de contenção (homologação): nullabilidade em CapturaLogin sob carga — v241</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Jun/2026</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Jun/2026</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>RNF04</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Concluída</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="56" t="inlineStr">
+        <is>
+          <t>20 tarefas — 20 concluídas</t>
         </is>
       </c>
     </row>
@@ -5483,7 +5567,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -5722,7 +5805,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="39.6" customHeight="1" s="38">
       <c r="A14" s="47" t="inlineStr">
         <is>
@@ -5794,7 +5876,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="1" t="n"/>
       <c r="B18" s="1" t="n"/>
@@ -5861,7 +5942,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -6181,7 +6261,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="47" t="inlineStr">
         <is>
@@ -6397,7 +6476,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="47" t="inlineStr">
         <is>
@@ -6583,7 +6661,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -7009,7 +7086,7 @@
     <row r="2">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Referência: CR-AASPAP01-001 · CR-AASPAP01-001 · REG-AASPAP01-001 §3.5</t>
+          <t>Referência: CR-AASPAP01-001 · CR-AASPAP01-002 · REG-AASPAP01-001 §3.5</t>
         </is>
       </c>
     </row>
@@ -7100,7 +7177,7 @@
     <row r="5">
       <c r="A5" s="55" t="inlineStr">
         <is>
-          <t>CR-AASPAP01-001</t>
+          <t>CR-AASPAP01-002</t>
         </is>
       </c>
       <c r="B5" s="55" t="inlineStr">
@@ -7139,7 +7216,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="57" t="inlineStr">
         <is>
@@ -7225,7 +7301,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
auditoria geral (Andamentos/AASPAP01): evidencias e registros alinhados ao GitLab
- remove prints do Azure DevOps (devops_andamentos_*): ferramenta de origem, dados divergentes do GitLab; mantidos apenas os prints gitlab_andamentos_* (conferem com o instance ao vivo)
- registros reconciliados (INDICE, GCO, ITP, REV-002, TAE, GEST)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mps-nivel-c/oficial/04_registros/AASP_Andamento-Processuais/GEST-AASPAP01_Planilha-de-Gestao-do-Projeto.xlsx
+++ b/mps-nivel-c/oficial/04_registros/AASP_Andamento-Processuais/GEST-AASPAP01_Planilha-de-Gestao-do-Projeto.xlsx
@@ -4717,7 +4717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" style="38" min="1" max="1"/>
@@ -5521,9 +5521,83 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="56" t="inlineStr">
-        <is>
-          <t>20 tarefas — 20 concluídas</t>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>T-21</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Correções na Controller da BotMax e prioridade de mensagem na fila</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Abr/2026</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Abr/2026</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>RF parceiras</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Concluída</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>T-22</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Verificação e atualização dos endpoints da API parceira BotMax</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Jun/2026</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>RF parceiras</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Em andamento</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="56" t="inlineStr">
+        <is>
+          <t>22 tarefas — 21 concluídas, 1 em andamento</t>
         </is>
       </c>
     </row>
@@ -5942,7 +6016,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -6262,7 +6335,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="47" t="inlineStr">
         <is>
@@ -6478,7 +6550,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="47" t="inlineStr">
         <is>

</xml_diff>